<commit_message>
Update automation test suite and project configuration
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/Login.xlsx
+++ b/src/test/resources/TestData/Login.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\HIEN\AT\DWR2510\src\test\resources\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ROSY\TSO\AT\DWR2510\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B874839-B7AA-45A1-BCC1-7CB57BF4F47C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B392C8ED-139F-4C27-BBB3-16CE85D18AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32700" yWindow="1290" windowWidth="21600" windowHeight="13215" xr2:uid="{E3BB357F-4007-4027-BE32-E1BA3BF329DF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3BB357F-4007-4027-BE32-E1BA3BF329DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>

</xml_diff>